<commit_message>
Remove parameter blocks and notes from the exercise workbooks
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HiyVPr15dFfxwtDW3Tiv76
</commit_message>
<xml_diff>
--- a/excel_bai_tap/bai2_ket_qua_thi_cuoi_khoa.xlsx
+++ b/excel_bai_tap/bai2_ket_qua_thi_cuoi_khoa.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="19">
   <si>
     <t xml:space="preserve">KẾT QUẢ THI CUỐI KHOÁ</t>
   </si>
@@ -55,28 +55,16 @@
     <t xml:space="preserve">Xếp hạng</t>
   </si>
   <si>
-    <t xml:space="preserve">Tham số (ô nhập)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Hiệp</t>
   </si>
   <si>
-    <t xml:space="preserve">KK cho HS nữ</t>
-  </si>
-  <si>
     <t xml:space="preserve">Nga</t>
   </si>
   <si>
     <t xml:space="preserve">x</t>
   </si>
   <si>
-    <t xml:space="preserve">KK cho HS nam</t>
-  </si>
-  <si>
     <t xml:space="preserve">Diễm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Điểm đậu (ĐTB &gt;=)</t>
   </si>
   <si>
     <t xml:space="preserve">Lâm</t>
@@ -100,7 +88,7 @@
     <numFmt numFmtId="165" formatCode="0.00"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -146,26 +134,13 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF0000FF"/>
-      <name val="Times New Roman"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor rgb="FFFFFF00"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -209,7 +184,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -220,10 +195,6 @@
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -239,18 +210,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -446,7 +405,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A2:M10"/>
+  <dimension ref="A2:J10"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -456,8 +415,6 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="8"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="8"/>
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -505,277 +462,256 @@
       <c r="J3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L3" s="3" t="s">
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="4"/>
-      <c r="D4" s="5" t="n">
+      <c r="C4" s="3"/>
+      <c r="D4" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="E4" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="F4" s="6" t="n">
-        <f aca="false">IF(C4="x",$M$4,$M$5)</f>
+      <c r="E4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <f aca="false">IF(C4="x",0.75,0.25)</f>
         <v>0.25</v>
       </c>
-      <c r="G4" s="5" t="n">
+      <c r="G4" s="4" t="n">
         <f aca="false">MIN(D4:E4)</f>
         <v>7</v>
       </c>
-      <c r="H4" s="7" t="n">
+      <c r="H4" s="6" t="n">
         <f aca="false">ROUND((D4+E4)/2+F4,1)</f>
         <v>8.3</v>
       </c>
-      <c r="I4" s="4" t="str">
-        <f aca="false">IF(H4&gt;=$M$6,"đậu","rớt")</f>
+      <c r="I4" s="3" t="str">
+        <f aca="false">IF(H4&gt;=5,"đậu","rớt")</f>
         <v>đậu</v>
       </c>
-      <c r="J4" s="4" t="n">
+      <c r="J4" s="3" t="n">
         <f aca="false">RANK(H4,$H$4:$H$10)</f>
         <v>2</v>
       </c>
-      <c r="L4" s="8" t="s">
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="M4" s="9" t="n">
+      <c r="D5" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <f aca="false">IF(C5="x",0.75,0.25)</f>
         <v>0.75</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="D5" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="E5" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="F5" s="6" t="n">
-        <f aca="false">IF(C5="x",$M$4,$M$5)</f>
-        <v>0.75</v>
-      </c>
-      <c r="G5" s="5" t="n">
+      <c r="G5" s="4" t="n">
         <f aca="false">MIN(D5:E5)</f>
         <v>6</v>
       </c>
-      <c r="H5" s="7" t="n">
+      <c r="H5" s="6" t="n">
         <f aca="false">ROUND((D5+E5)/2+F5,1)</f>
         <v>7.3</v>
       </c>
-      <c r="I5" s="4" t="str">
-        <f aca="false">IF(H5&gt;=$M$6,"đậu","rớt")</f>
+      <c r="I5" s="3" t="str">
+        <f aca="false">IF(H5&gt;=5,"đậu","rớt")</f>
         <v>đậu</v>
       </c>
-      <c r="J5" s="4" t="n">
+      <c r="J5" s="3" t="n">
         <f aca="false">RANK(H5,$H$4:$H$10)</f>
         <v>4</v>
       </c>
-      <c r="L5" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="M5" s="9" t="n">
-        <v>0.25</v>
-      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="n">
+      <c r="A6" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="D6" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="E6" s="5" t="n">
+      <c r="B6" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E6" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="F6" s="6" t="n">
-        <f aca="false">IF(C6="x",$M$4,$M$5)</f>
+      <c r="F6" s="5" t="n">
+        <f aca="false">IF(C6="x",0.75,0.25)</f>
         <v>0.75</v>
       </c>
-      <c r="G6" s="5" t="n">
+      <c r="G6" s="4" t="n">
         <f aca="false">MIN(D6:E6)</f>
         <v>6</v>
       </c>
-      <c r="H6" s="7" t="n">
+      <c r="H6" s="6" t="n">
         <f aca="false">ROUND((D6+E6)/2+F6,1)</f>
         <v>7.3</v>
       </c>
-      <c r="I6" s="4" t="str">
-        <f aca="false">IF(H6&gt;=$M$6,"đậu","rớt")</f>
+      <c r="I6" s="3" t="str">
+        <f aca="false">IF(H6&gt;=5,"đậu","rớt")</f>
         <v>đậu</v>
       </c>
-      <c r="J6" s="4" t="n">
+      <c r="J6" s="3" t="n">
         <f aca="false">RANK(H6,$H$4:$H$10)</f>
         <v>4</v>
       </c>
-      <c r="L6" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="M6" s="10" t="n">
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="3"/>
+      <c r="D7" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="E7" s="4" t="n">
         <v>5</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C7" s="4"/>
-      <c r="D7" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="E7" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="F7" s="6" t="n">
-        <f aca="false">IF(C7="x",$M$4,$M$5)</f>
+      <c r="F7" s="5" t="n">
+        <f aca="false">IF(C7="x",0.75,0.25)</f>
         <v>0.25</v>
       </c>
-      <c r="G7" s="5" t="n">
+      <c r="G7" s="4" t="n">
         <f aca="false">MIN(D7:E7)</f>
         <v>4</v>
       </c>
-      <c r="H7" s="7" t="n">
+      <c r="H7" s="6" t="n">
         <f aca="false">ROUND((D7+E7)/2+F7,1)</f>
         <v>4.8</v>
       </c>
-      <c r="I7" s="4" t="str">
-        <f aca="false">IF(H7&gt;=$M$6,"đậu","rớt")</f>
+      <c r="I7" s="3" t="str">
+        <f aca="false">IF(H7&gt;=5,"đậu","rớt")</f>
         <v>rớt</v>
       </c>
-      <c r="J7" s="4" t="n">
+      <c r="J7" s="3" t="n">
         <f aca="false">RANK(H7,$H$4:$H$10)</f>
         <v>7</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="n">
+      <c r="A8" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="D8" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="E8" s="5" t="n">
+      <c r="B8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E8" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="F8" s="6" t="n">
-        <f aca="false">IF(C8="x",$M$4,$M$5)</f>
+      <c r="F8" s="5" t="n">
+        <f aca="false">IF(C8="x",0.75,0.25)</f>
         <v>0.75</v>
       </c>
-      <c r="G8" s="5" t="n">
+      <c r="G8" s="4" t="n">
         <f aca="false">MIN(D8:E8)</f>
         <v>7</v>
       </c>
-      <c r="H8" s="7" t="n">
+      <c r="H8" s="6" t="n">
         <f aca="false">ROUND((D8+E8)/2+F8,1)</f>
         <v>8.3</v>
       </c>
-      <c r="I8" s="4" t="str">
-        <f aca="false">IF(H8&gt;=$M$6,"đậu","rớt")</f>
+      <c r="I8" s="3" t="str">
+        <f aca="false">IF(H8&gt;=5,"đậu","rớt")</f>
         <v>đậu</v>
       </c>
-      <c r="J8" s="4" t="n">
+      <c r="J8" s="3" t="n">
         <f aca="false">RANK(H8,$H$4:$H$10)</f>
         <v>2</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="n">
+      <c r="A9" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="C9" s="4"/>
-      <c r="D9" s="5" t="n">
+      <c r="B9" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="3"/>
+      <c r="D9" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="E9" s="5" t="n">
+      <c r="E9" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="F9" s="6" t="n">
-        <f aca="false">IF(C9="x",$M$4,$M$5)</f>
+      <c r="F9" s="5" t="n">
+        <f aca="false">IF(C9="x",0.75,0.25)</f>
         <v>0.25</v>
       </c>
-      <c r="G9" s="5" t="n">
+      <c r="G9" s="4" t="n">
         <f aca="false">MIN(D9:E9)</f>
         <v>6</v>
       </c>
-      <c r="H9" s="7" t="n">
+      <c r="H9" s="6" t="n">
         <f aca="false">ROUND((D9+E9)/2+F9,1)</f>
         <v>7.3</v>
       </c>
-      <c r="I9" s="4" t="str">
-        <f aca="false">IF(H9&gt;=$M$6,"đậu","rớt")</f>
+      <c r="I9" s="3" t="str">
+        <f aca="false">IF(H9&gt;=5,"đậu","rớt")</f>
         <v>đậu</v>
       </c>
-      <c r="J9" s="4" t="n">
+      <c r="J9" s="3" t="n">
         <f aca="false">RANK(H9,$H$4:$H$10)</f>
         <v>4</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="D10" s="5" t="n">
+      <c r="A10" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="E10" s="5" t="n">
+      <c r="E10" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="F10" s="6" t="n">
-        <f aca="false">IF(C10="x",$M$4,$M$5)</f>
+      <c r="F10" s="5" t="n">
+        <f aca="false">IF(C10="x",0.75,0.25)</f>
         <v>0.75</v>
       </c>
-      <c r="G10" s="5" t="n">
+      <c r="G10" s="4" t="n">
         <f aca="false">MIN(D10:E10)</f>
         <v>8</v>
       </c>
-      <c r="H10" s="7" t="n">
+      <c r="H10" s="6" t="n">
         <f aca="false">ROUND((D10+E10)/2+F10,1)</f>
         <v>9.8</v>
       </c>
-      <c r="I10" s="4" t="str">
-        <f aca="false">IF(H10&gt;=$M$6,"đậu","rớt")</f>
+      <c r="I10" s="3" t="str">
+        <f aca="false">IF(H10&gt;=5,"đậu","rớt")</f>
         <v>đậu</v>
       </c>
-      <c r="J10" s="4" t="n">
+      <c r="J10" s="3" t="n">
         <f aca="false">RANK(H10,$H$4:$H$10)</f>
         <v>1</v>
       </c>

</xml_diff>